<commit_message>
Show which JMISC pin each of the signals are on
</commit_message>
<xml_diff>
--- a/Documents/uno_q_pin_info.xlsx
+++ b/Documents/uno_q_pin_info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\github\Arduino_UNO_Q\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{811797C3-C53B-47BE-8BFB-88439DECF1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9067DA-1EAA-4203-A4C0-D5EB1065A6E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3405" yWindow="1125" windowWidth="30480" windowHeight="19215" xr2:uid="{E4BC628E-A193-46B6-8015-32829E9A0B6A}"/>
+    <workbookView xWindow="-30" yWindow="1335" windowWidth="24690" windowHeight="19215" xr2:uid="{E4BC628E-A193-46B6-8015-32829E9A0B6A}"/>
   </bookViews>
   <sheets>
     <sheet name="Alternate functions" sheetId="4" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2554" uniqueCount="607">
   <si>
     <t>PE2</t>
   </si>
@@ -1829,9 +1829,6 @@
     <t>D24/JSPI</t>
   </si>
   <si>
-    <t>JMISC</t>
-  </si>
-  <si>
     <t>LED3_R</t>
   </si>
   <si>
@@ -1875,6 +1872,81 @@
   </si>
   <si>
     <t>3,6</t>
+  </si>
+  <si>
+    <t>JMISC_1</t>
+  </si>
+  <si>
+    <t>JMISC_2</t>
+  </si>
+  <si>
+    <t>JMISC_3</t>
+  </si>
+  <si>
+    <t>JMISC_4</t>
+  </si>
+  <si>
+    <t>JMISC_5</t>
+  </si>
+  <si>
+    <t>JMISC_6</t>
+  </si>
+  <si>
+    <t>JMISC_7</t>
+  </si>
+  <si>
+    <t>JMISC_8</t>
+  </si>
+  <si>
+    <t>JMISC_9</t>
+  </si>
+  <si>
+    <t>JMISC_10</t>
+  </si>
+  <si>
+    <t>JMISC_11</t>
+  </si>
+  <si>
+    <t>JMISC_12</t>
+  </si>
+  <si>
+    <t>JMISC_13</t>
+  </si>
+  <si>
+    <t>JMISC_14</t>
+  </si>
+  <si>
+    <t>JMISC_15</t>
+  </si>
+  <si>
+    <t>JMISC_16</t>
+  </si>
+  <si>
+    <t>JMISC_17</t>
+  </si>
+  <si>
+    <t>JMISC_18</t>
+  </si>
+  <si>
+    <t>JMISC_19</t>
+  </si>
+  <si>
+    <t>JMISC_20</t>
+  </si>
+  <si>
+    <t>JMISC_21</t>
+  </si>
+  <si>
+    <t>JMISC_22</t>
+  </si>
+  <si>
+    <t>JMISC_23</t>
+  </si>
+  <si>
+    <t>JMISC_24</t>
+  </si>
+  <si>
+    <t>JMISC_25</t>
   </si>
 </sst>
 </file>
@@ -2061,23 +2133,23 @@
     <tableColumn id="1" xr3:uid="{5D3DC2F8-BE01-4770-90D9-5E86DD3515C5}" name="Arduino Pin" dataDxfId="19"/>
     <tableColumn id="2" xr3:uid="{4DF36108-303C-4552-A60D-FC0595910492}" name="usage" dataDxfId="18"/>
     <tableColumn id="3" xr3:uid="{5811D300-4E1E-42C2-907B-C9CB2B8C6F0D}" name="Port" dataDxfId="17"/>
-    <tableColumn id="20" xr3:uid="{A25879C6-B528-4988-8519-F72B117DA08E}" name="Tolerant" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{74BE88FF-5CE3-461F-A123-4B7D553806F5}" name="AF0" dataDxfId="16"/>
-    <tableColumn id="5" xr3:uid="{3954F4BC-2868-47FB-8E8F-45EC4574FF90}" name="AF1" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{1BD10078-5CBC-474B-9DA3-0ED9E02640CC}" name="AF2" dataDxfId="14"/>
-    <tableColumn id="7" xr3:uid="{BAF4C0D9-F5FC-4BD9-A3AD-6468389DB9A7}" name="AF3" dataDxfId="13"/>
-    <tableColumn id="8" xr3:uid="{5218359D-232A-41D1-B9D8-5007ACB972A9}" name="AF4" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{02FE55B4-3775-4437-94F3-8969261B600D}" name="AF5" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{9CB95CDE-98DB-4DC7-BC12-24E205076715}" name="AF6" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{E1BCDB17-8F81-4C96-8F69-5E6B75135343}" name="AF7" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{D3885D50-853B-47B8-9AB1-55C573D700A6}" name="AF8" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{8D8F5E86-F9E1-4B5B-A61E-708EC27FEA0C}" name="AF9" dataDxfId="7"/>
-    <tableColumn id="14" xr3:uid="{FB09A257-B323-4805-A01A-AE2A1C949B27}" name="AF10" dataDxfId="6"/>
-    <tableColumn id="15" xr3:uid="{6D47C5BB-E8B8-402F-B6DA-1A62C563C332}" name="AF11" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{A2BF269C-9E8F-4F38-899F-A0607D6FD01A}" name="AF12" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{60F5BB27-9C71-46A2-8A33-34B2F87EEFB2}" name="AF13" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{D03D8DB4-217F-4E09-8CE9-81318E9E3979}" name="AF14" dataDxfId="2"/>
-    <tableColumn id="19" xr3:uid="{D043E6A3-4209-4229-85F5-7672216074E8}" name="AF15" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{A25879C6-B528-4988-8519-F72B117DA08E}" name="Tolerant" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{74BE88FF-5CE3-461F-A123-4B7D553806F5}" name="AF0" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{3954F4BC-2868-47FB-8E8F-45EC4574FF90}" name="AF1" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{1BD10078-5CBC-474B-9DA3-0ED9E02640CC}" name="AF2" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{BAF4C0D9-F5FC-4BD9-A3AD-6468389DB9A7}" name="AF3" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{5218359D-232A-41D1-B9D8-5007ACB972A9}" name="AF4" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{02FE55B4-3775-4437-94F3-8969261B600D}" name="AF5" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{9CB95CDE-98DB-4DC7-BC12-24E205076715}" name="AF6" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{E1BCDB17-8F81-4C96-8F69-5E6B75135343}" name="AF7" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{D3885D50-853B-47B8-9AB1-55C573D700A6}" name="AF8" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{8D8F5E86-F9E1-4B5B-A61E-708EC27FEA0C}" name="AF9" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{FB09A257-B323-4805-A01A-AE2A1C949B27}" name="AF10" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{6D47C5BB-E8B8-402F-B6DA-1A62C563C332}" name="AF11" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{A2BF269C-9E8F-4F38-899F-A0607D6FD01A}" name="AF12" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{60F5BB27-9C71-46A2-8A33-34B2F87EEFB2}" name="AF13" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{D03D8DB4-217F-4E09-8CE9-81318E9E3979}" name="AF14" dataDxfId="1"/>
+    <tableColumn id="19" xr3:uid="{D043E6A3-4209-4229-85F5-7672216074E8}" name="AF15" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2438,7 +2510,7 @@
         <v>52</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>53</v>
@@ -2500,7 +2572,7 @@
         <v>179</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>1</v>
@@ -2562,7 +2634,7 @@
         <v>172</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>1</v>
@@ -2624,7 +2696,7 @@
         <v>158</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>159</v>
@@ -2686,7 +2758,7 @@
         <v>33</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>1</v>
@@ -2748,7 +2820,7 @@
         <v>131</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>1</v>
@@ -2810,7 +2882,7 @@
         <v>127</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>1</v>
@@ -2872,7 +2944,7 @@
         <v>34</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>1</v>
@@ -2934,7 +3006,7 @@
         <v>35</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>1</v>
@@ -2996,7 +3068,7 @@
         <v>163</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>164</v>
@@ -3058,7 +3130,7 @@
         <v>184</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>1</v>
@@ -3120,7 +3192,7 @@
         <v>187</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>1</v>
@@ -3182,7 +3254,7 @@
         <v>206</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>207</v>
@@ -3244,7 +3316,7 @@
         <v>202</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -3300,13 +3372,13 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>199</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>1</v>
@@ -3368,7 +3440,7 @@
         <v>27</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>1</v>
@@ -3430,7 +3502,7 @@
         <v>28</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>92</v>
@@ -3492,7 +3564,7 @@
         <v>29</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>97</v>
@@ -3554,7 +3626,7 @@
         <v>30</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>104</v>
@@ -3616,7 +3688,7 @@
         <v>20</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>212</v>
@@ -3678,7 +3750,7 @@
         <v>19</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>1</v>
@@ -3740,7 +3812,7 @@
         <v>193</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>1</v>
@@ -3802,7 +3874,7 @@
         <v>191</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>1</v>
@@ -3864,7 +3936,7 @@
         <v>21</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>1</v>
@@ -3926,7 +3998,7 @@
         <v>22</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>1</v>
@@ -3988,7 +4060,7 @@
         <v>240</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>1</v>
@@ -4044,13 +4116,13 @@
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>567</v>
+        <v>582</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>218</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>92</v>
@@ -4106,13 +4178,13 @@
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>567</v>
+        <v>583</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>241</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>242</v>
@@ -4168,13 +4240,13 @@
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>567</v>
+        <v>584</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>221</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>97</v>
@@ -4230,13 +4302,13 @@
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>567</v>
+        <v>585</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>0</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>263</v>
@@ -4292,13 +4364,13 @@
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>567</v>
+        <v>586</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>224</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>104</v>
@@ -4354,13 +4426,13 @@
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>567</v>
+        <v>587</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>212</v>
@@ -4416,13 +4488,13 @@
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>567</v>
+        <v>588</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>226</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>212</v>
@@ -4478,13 +4550,13 @@
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>567</v>
+        <v>589</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>242</v>
@@ -4540,13 +4612,13 @@
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>567</v>
+        <v>590</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>3</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>230</v>
@@ -4602,13 +4674,13 @@
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>567</v>
+        <v>591</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>5</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>236</v>
@@ -4664,13 +4736,13 @@
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>567</v>
+        <v>592</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>318</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>1</v>
@@ -4726,13 +4798,13 @@
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>567</v>
+        <v>593</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>43</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>1</v>
@@ -4788,13 +4860,13 @@
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>567</v>
+        <v>594</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>320</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>1</v>
@@ -4850,13 +4922,13 @@
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>567</v>
+        <v>595</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>44</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>1</v>
@@ -4912,13 +4984,13 @@
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>567</v>
+        <v>596</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>321</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>1</v>
@@ -4974,13 +5046,13 @@
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>567</v>
+        <v>597</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>39</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>1</v>
@@ -5036,13 +5108,13 @@
         <v>41</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>567</v>
+        <v>598</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>252</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>1</v>
@@ -5098,13 +5170,13 @@
         <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>567</v>
+        <v>599</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>40</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>1</v>
@@ -5160,13 +5232,13 @@
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>567</v>
+        <v>600</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>319</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>1</v>
@@ -5222,13 +5294,13 @@
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>567</v>
+        <v>601</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>26</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>1</v>
@@ -5284,13 +5356,13 @@
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>567</v>
+        <v>602</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>251</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>1</v>
@@ -5346,13 +5418,13 @@
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>567</v>
+        <v>603</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>23</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>1</v>
@@ -5408,13 +5480,13 @@
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>567</v>
+        <v>604</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>110</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>111</v>
@@ -5470,13 +5542,13 @@
         <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>567</v>
+        <v>605</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>24</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>74</v>
@@ -5532,13 +5604,13 @@
         <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>567</v>
+        <v>606</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>120</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>121</v>
@@ -5594,13 +5666,13 @@
         <v>50</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>568</v>
+        <v>567</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>305</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>1</v>
@@ -5656,13 +5728,13 @@
         <v>51</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>306</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>1</v>
@@ -5718,13 +5790,13 @@
         <v>52</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>307</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>1</v>
@@ -5780,13 +5852,13 @@
         <v>53</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>308</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>1</v>
@@ -5842,13 +5914,13 @@
         <v>54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>309</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>1</v>
@@ -5904,13 +5976,13 @@
         <v>55</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>310</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>1</v>
@@ -5966,13 +6038,13 @@
         <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>1</v>
@@ -6028,13 +6100,13 @@
         <v>57</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>9</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>1</v>
@@ -6090,13 +6162,13 @@
         <v>58</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>10</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>1</v>
@@ -6152,13 +6224,13 @@
         <v>59</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>1</v>
@@ -6214,13 +6286,13 @@
         <v>60</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>12</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>1</v>
@@ -6276,13 +6348,13 @@
         <v>61</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>1</v>
@@ -6338,13 +6410,13 @@
         <v>62</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C64" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>1</v>
@@ -6400,13 +6472,13 @@
         <v>63</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C65" s="1" t="s">
         <v>15</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>1</v>
@@ -6462,13 +6534,13 @@
         <v>64</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C66" s="1" t="s">
         <v>16</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>1</v>
@@ -6524,13 +6596,13 @@
         <v>65</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C67" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>1</v>
@@ -6586,13 +6658,13 @@
         <v>66</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>1</v>
@@ -6648,13 +6720,13 @@
         <v>67</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>291</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>1</v>
@@ -6710,13 +6782,13 @@
         <v>68</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>25</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>1</v>
@@ -6772,13 +6844,13 @@
         <v>69</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>577</v>
+        <v>576</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>298</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>1</v>
@@ -6834,7 +6906,7 @@
         <v>135</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>136</v>
@@ -6890,7 +6962,7 @@
         <v>138</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>139</v>
@@ -6946,7 +7018,7 @@
         <v>142</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>143</v>
@@ -7002,7 +7074,7 @@
         <v>115</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>1</v>
@@ -7058,7 +7130,7 @@
         <v>196</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>1</v>
@@ -7114,7 +7186,7 @@
         <v>168</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>1</v>
@@ -7170,7 +7242,7 @@
         <v>229</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>230</v>
@@ -7226,7 +7298,7 @@
         <v>232</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>1</v>
@@ -7282,7 +7354,7 @@
         <v>235</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E80" s="1" t="s">
         <v>236</v>
@@ -7338,7 +7410,7 @@
         <v>6</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E81" s="1" t="s">
         <v>1</v>
@@ -7394,7 +7466,7 @@
         <v>237</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E82" s="1" t="s">
         <v>1</v>
@@ -7450,7 +7522,7 @@
         <v>238</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E83" s="1" t="s">
         <v>1</v>
@@ -7506,7 +7578,7 @@
         <v>31</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E84" s="1" t="s">
         <v>1</v>
@@ -7562,7 +7634,7 @@
         <v>32</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E85" s="1" t="s">
         <v>1</v>
@@ -7618,7 +7690,7 @@
         <v>239</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E86" s="1" t="s">
         <v>1</v>
@@ -7674,7 +7746,7 @@
         <v>253</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E87" s="1" t="s">
         <v>1</v>
@@ -7730,7 +7802,7 @@
         <v>255</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E88" s="1" t="s">
         <v>1</v>
@@ -7786,7 +7858,7 @@
         <v>256</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E89" s="1" t="s">
         <v>1</v>
@@ -7842,7 +7914,7 @@
         <v>257</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E90" s="1" t="s">
         <v>1</v>
@@ -7898,7 +7970,7 @@
         <v>258</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E91" s="1" t="s">
         <v>1</v>
@@ -7954,7 +8026,7 @@
         <v>259</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E92" s="1" t="s">
         <v>1</v>
@@ -8010,7 +8082,7 @@
         <v>244</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E93" s="1" t="s">
         <v>1</v>
@@ -8066,7 +8138,7 @@
         <v>246</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E94" s="1" t="s">
         <v>1</v>
@@ -8122,7 +8194,7 @@
         <v>247</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>1</v>
@@ -8178,7 +8250,7 @@
         <v>248</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E96" s="1" t="s">
         <v>1</v>
@@ -8234,7 +8306,7 @@
         <v>250</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E97" s="1" t="s">
         <v>1</v>
@@ -8290,7 +8362,7 @@
         <v>260</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E98" s="1" t="s">
         <v>1</v>
@@ -8346,7 +8418,7 @@
         <v>262</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E99" s="1" t="s">
         <v>1</v>
@@ -8402,7 +8474,7 @@
         <v>46</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E100" s="1" t="s">
         <v>1</v>
@@ -8458,7 +8530,7 @@
         <v>47</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E101" s="1" t="s">
         <v>1</v>
@@ -8514,7 +8586,7 @@
         <v>48</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E102" s="1" t="s">
         <v>1</v>
@@ -8570,7 +8642,7 @@
         <v>49</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E103" s="1" t="s">
         <v>1</v>
@@ -8626,7 +8698,7 @@
         <v>50</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E104" s="1" t="s">
         <v>1</v>
@@ -8682,7 +8754,7 @@
         <v>51</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E105" s="1" t="s">
         <v>1</v>
@@ -8738,7 +8810,7 @@
         <v>45</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E106" s="1" t="s">
         <v>1</v>
@@ -8794,7 +8866,7 @@
         <v>36</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E107" s="1" t="s">
         <v>1</v>
@@ -8850,7 +8922,7 @@
         <v>37</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E108" s="1" t="s">
         <v>1</v>
@@ -8906,7 +8978,7 @@
         <v>38</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E109" s="1" t="s">
         <v>1</v>
@@ -8962,7 +9034,7 @@
         <v>41</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E110" s="1" t="s">
         <v>1</v>
@@ -9018,7 +9090,7 @@
         <v>42</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E111" s="1" t="s">
         <v>1</v>
@@ -9074,7 +9146,7 @@
         <v>286</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E112" s="1" t="s">
         <v>1</v>
@@ -9130,7 +9202,7 @@
         <v>288</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E113" s="1" t="s">
         <v>1</v>
@@ -9186,7 +9258,7 @@
         <v>290</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E114" s="1" t="s">
         <v>1</v>
@@ -9242,7 +9314,7 @@
         <v>292</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E115" s="1" t="s">
         <v>1</v>
@@ -9298,7 +9370,7 @@
         <v>293</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E116" s="1" t="s">
         <v>1</v>
@@ -9354,7 +9426,7 @@
         <v>277</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E117" s="1" t="s">
         <v>1</v>
@@ -9410,7 +9482,7 @@
         <v>278</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E118" s="1" t="s">
         <v>1</v>
@@ -9466,7 +9538,7 @@
         <v>279</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E119" s="1" t="s">
         <v>1</v>
@@ -9522,7 +9594,7 @@
         <v>280</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E120" s="1" t="s">
         <v>1</v>
@@ -9578,7 +9650,7 @@
         <v>281</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E121" s="1" t="s">
         <v>1</v>
@@ -9634,7 +9706,7 @@
         <v>282</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E122" s="1" t="s">
         <v>1</v>
@@ -9690,7 +9762,7 @@
         <v>283</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E123" s="1" t="s">
         <v>1</v>
@@ -9746,7 +9818,7 @@
         <v>284</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E124" s="1" t="s">
         <v>1</v>
@@ -9802,7 +9874,7 @@
         <v>294</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E125" s="1" t="s">
         <v>1</v>
@@ -9858,7 +9930,7 @@
         <v>295</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E126" s="1" t="s">
         <v>1</v>
@@ -9914,7 +9986,7 @@
         <v>296</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E127" s="1" t="s">
         <v>1</v>
@@ -9970,7 +10042,7 @@
         <v>299</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E128" s="1" t="s">
         <v>1</v>
@@ -10026,7 +10098,7 @@
         <v>300</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E129" s="1" t="s">
         <v>1</v>
@@ -10082,7 +10154,7 @@
         <v>301</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E130" s="1" t="s">
         <v>1</v>
@@ -10138,7 +10210,7 @@
         <v>302</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E131" s="1" t="s">
         <v>1</v>
@@ -10194,7 +10266,7 @@
         <v>303</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E132" s="1" t="s">
         <v>1</v>
@@ -10250,7 +10322,7 @@
         <v>304</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E133" s="1" t="s">
         <v>1</v>
@@ -10306,7 +10378,7 @@
         <v>311</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E134" s="1" t="s">
         <v>1</v>
@@ -10362,7 +10434,7 @@
         <v>312</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E135" s="1" t="s">
         <v>1</v>
@@ -10418,7 +10490,7 @@
         <v>314</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E136" s="1" t="s">
         <v>1</v>
@@ -10474,7 +10546,7 @@
         <v>316</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="E137" s="1" t="s">
         <v>1</v>

</xml_diff>